<commit_message>
corpus: rj002 declares the K0 its own tag names
apply_tag_k0 writes main!D16 from the page's tag, so a row that gains a tag
gains the declared K0. RJ-2's tag was written after the file was last built, and
verify_rebuild caught the file and the builder disagreeing. The solve is
unaffected -- the run took k0 = 1 from the tag either way -- but the initial
stress has to live in the FILE or the locked factor is reproducible from the
suite and from nothing a user would open.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XjjT2aBxw8gY7EFdpoUcpj
</commit_message>
<xml_diff>
--- a/docs/verification/files/rocscience/joints/rj002.xlsx
+++ b/docs/verification/files/rocscience/joints/rj002.xlsx
@@ -3374,7 +3374,9 @@
       <c r="G16" t="s">
         <v>34</v>
       </c>
-      <c r="D16"/>
+      <c r="D16">
+        <v>1.0</v>
+      </c>
     </row>
     <row r="17" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B17" s="1"/>

</xml_diff>